<commit_message>
No diff provided; unable to summarize changes
</commit_message>
<xml_diff>
--- a/J30/Output_files/MHE_Journal_Inbound_results.xlsx
+++ b/J30/Output_files/MHE_Journal_Inbound_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,12 +488,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DEI-2026-06-29-02-27-36-095-RPKC</t>
+          <t>DEI-2026-07-29-13-07-26-803-saQH</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>00081062920260003101</t>
+          <t>00000010379092983216</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -513,12 +513,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>vgana3</t>
+          <t>asure2</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-06-29T02:28:18.796591</t>
+          <t>2026-07-29T13:08:15.492036</t>
         </is>
       </c>
     </row>
@@ -535,12 +535,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DEI-2026-06-29-02-27-46-732-9Nqp</t>
+          <t>DEI-2026-07-29-13-07-30-053-owOQ</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>00081062920260003101</t>
+          <t>00000010379092983216</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>PTW_DEI_AllocationCreated</t>
+          <t>GoodsholderMeasured</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -560,12 +560,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>vgana3</t>
+          <t>asure2</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-06-29T02:28:18.800368</t>
+          <t>2026-07-29T13:08:15.492036</t>
         </is>
       </c>
     </row>
@@ -582,12 +582,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DEI-2026-06-29-02-27-36-480-cPeH</t>
+          <t>DEI-2026-07-29-13-07-32-056-Lihh</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>00081062920260003102</t>
+          <t>00000010379092983216</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>GoodsholderAnnounced</t>
+          <t>PTW_DEI_AllocationCreated</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -607,12 +607,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>vgana3</t>
+          <t>asure2</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-06-29T02:28:18.800368</t>
+          <t>2026-07-29T13:08:15.492079</t>
         </is>
       </c>
     </row>
@@ -629,12 +629,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DEI-2026-06-29-02-27-48-016-WO9z</t>
+          <t>DEI-2026-07-29-13-27-41-811-Zckl</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>00081062920260003102</t>
+          <t>00000010379092983216</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -644,22 +644,210 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>PutawayTaskResult</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>vgana3</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-07-29T13:28:25.565806</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1081</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>DEI-2026-07-29-13-07-29-272-z4Sg</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>00000010585288239549</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>GoodsholderMeasured</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>asure2</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-07-29T13:08:15.492036</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1081</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>DEI-2026-07-29-13-07-25-990-DXHJ</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>00000010585288239549</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>GoodsholderAnnounced</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>vgana3</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-07-29T13:14:05.506055</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1081</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DEI-2026-07-29-13-13-20-939-MNJn</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>00000010585288239549</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>PTW_DEI_AllocationCreated</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>COMPLETED</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>vgana3</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-06-29T02:28:18.803171</t>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-07-29T13:14:05.506145</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1081</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DEI-2026-07-29-13-27-40-884-BZQ3</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>00000010585288239549</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PutawayTaskResult</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>vgana3</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-07-29T13:28:25.566131</t>
         </is>
       </c>
     </row>

</xml_diff>